<commit_message>
Complete Sonelgaz chatbot prototype and RAG integration
</commit_message>
<xml_diff>
--- a/data/dataset_facture.xlsx
+++ b/data/dataset_facture.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2035"/>
+  <dimension ref="A1:F2055"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65400,6 +65400,646 @@
       <c r="E2035" t="inlineStr"/>
       <c r="F2035" t="inlineStr"/>
     </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>majatnich la facture ta3i</t>
+        </is>
+      </c>
+      <c r="D2036" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2036" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2036" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>mazal ma waslatnich facture ta3i</t>
+        </is>
+      </c>
+      <c r="D2037" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2037" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2037" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>la facture ta3i mazal ma jatnich</t>
+        </is>
+      </c>
+      <c r="D2038" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2038" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2038" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>win rah la facture ta3i</t>
+        </is>
+      </c>
+      <c r="D2039" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2039" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2039" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>la facture ta3i ma wslatch</t>
+        </is>
+      </c>
+      <c r="D2040" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2040" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2040" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>facture ta3 had chhar ma waslatnich</t>
+        </is>
+      </c>
+      <c r="D2041" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2041" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2041" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>mazal نستنى la facture ta3i</t>
+        </is>
+      </c>
+      <c r="D2042" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2042" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2042" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>ma banetlich la facture ta3i</t>
+        </is>
+      </c>
+      <c r="D2043" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2043" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2043" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>ma l9itch facture ta3i had chhar</t>
+        </is>
+      </c>
+      <c r="D2044" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2044" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2044" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>la facture ta3i ma jatnich</t>
+        </is>
+      </c>
+      <c r="D2045" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2045" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2045" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>had chhar ma جاتنيش la facture</t>
+        </is>
+      </c>
+      <c r="D2046" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2046" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2046" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>maزال ما جاتنيش facture Sonelgaz</t>
+        </is>
+      </c>
+      <c r="D2047" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2047" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2047" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>facture ta3i ma wasletlich</t>
+        </is>
+      </c>
+      <c r="D2048" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2048" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2048" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>win hiya facture ta3i</t>
+        </is>
+      </c>
+      <c r="D2049" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2049" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2049" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>ma waslatnich facture had chhar</t>
+        </is>
+      </c>
+      <c r="D2050" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2050" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2050" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>la facture ma banetlich had chhar</t>
+        </is>
+      </c>
+      <c r="D2051" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2051" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2051" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>mazal نستنى facture ta3i</t>
+        </is>
+      </c>
+      <c r="D2052" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2052" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2052" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>facture ta3i ma wslatlich</t>
+        </is>
+      </c>
+      <c r="D2053" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2053" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2053" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>ma jatnich la facture cette fois</t>
+        </is>
+      </c>
+      <c r="D2054" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2054" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2054" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>FACTURE</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>bill_not_received</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>la facture ta3 had chhar mazal ma jatnich</t>
+        </is>
+      </c>
+      <c r="D2055" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E2055" t="inlineStr">
+        <is>
+          <t>Si vous n'avez pas reçu votre facture, vous pouvez vous présenter à votre agence commerciale avec une ancienne facture de consommation.</t>
+        </is>
+      </c>
+      <c r="F2055" t="inlineStr">
+        <is>
+          <t>scenario_facture.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>